<commit_message>
Fusionner les cibles dupliquées et enrichir l'affichage des mappings CDA/FHIR b3d8c7005fa215effe86da409fc38cf2fb233b31
</commit_message>
<xml_diff>
--- a/fix-mapping-entete-duplicate-targets/ig/FRCustodianLMCDAFHIR.xlsx
+++ b/fix-mapping-entete-duplicate-targets/ig/FRCustodianLMCDAFHIR.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="49">
   <si>
     <t>Property</t>
   </si>
@@ -62,7 +62,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-02T10:43:57+00:00</t>
+    <t>2026-09-02T12:54:48+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -119,6 +119,9 @@
   </si>
   <si>
     <t>FRLMHeaderDocument.custodian</t>
+  </si>
+  <si>
+    <t>FRLMOrganisation</t>
   </si>
   <si>
     <t>equivalent</t>
@@ -457,12 +460,14 @@
       <c r="A3" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" t="s" s="2">
+        <v>34</v>
+      </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2"/>
     </row>
@@ -495,7 +500,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="2">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s" s="2">
         <v>31</v>
@@ -504,7 +509,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -512,53 +517,53 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -600,7 +605,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -610,12 +615,14 @@
       <c r="A3" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" t="s" s="2">
+        <v>34</v>
+      </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E3" s="2"/>
     </row>

</xml_diff>